<commit_message>
Add cost-base note to model Summary tab
Co-authored-by: JoaoTavarees <JoaoTavarees@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/luca_chief_of_staff_case/deliverables/Luca_Step1_Financial_Model.xlsx
+++ b/luca_chief_of_staff_case/deliverables/Luca_Step1_Financial_Model.xlsx
@@ -725,7 +725,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -1036,6 +1036,57 @@
       <c r="C22" s="2" t="n"/>
       <c r="D22" s="2" t="n"/>
       <c r="E22" s="2" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="n"/>
+      <c r="B23" s="2" t="n"/>
+      <c r="C23" s="2" t="n"/>
+      <c r="D23" s="2" t="n"/>
+      <c r="E23" s="2" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n"/>
+      <c r="B24" s="10" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="n"/>
+      <c r="D24" s="2" t="n"/>
+      <c r="E24" s="2" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="n"/>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>The case cost base covers only the 25 new hires, overhead and G&amp;A, so Luca generates cash every month</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="n"/>
+      <c r="D25" s="2" t="n"/>
+      <c r="E25" s="2" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n"/>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>and runway is not a constraint. Next step before the board: add Luca's existing cost base (current team,</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="n"/>
+      <c r="D26" s="2" t="n"/>
+      <c r="E26" s="2" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="n"/>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>marketing, technology) to the model. That is where runway and the loan decision become relevant.</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="n"/>
+      <c r="D27" s="2" t="n"/>
+      <c r="E27" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Reword runway note in deck and model Summary
Co-authored-by: JoaoTavarees <JoaoTavarees@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/luca_chief_of_staff_case/deliverables/Luca_Step1_Financial_Model.xlsx
+++ b/luca_chief_of_staff_case/deliverables/Luca_Step1_Financial_Model.xlsx
@@ -1059,7 +1059,7 @@
       <c r="A25" s="2" t="n"/>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>The case cost base covers only the 25 new hires, overhead and G&amp;A, so Luca generates cash every month</t>
+          <t>Runway isn't a real constraint in this case. Luca generates $0.9–1.5M of cash every month (about $13.6M</t>
         </is>
       </c>
       <c r="C25" s="2" t="n"/>
@@ -1070,7 +1070,7 @@
       <c r="A26" s="2" t="n"/>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>and runway is not a constraint. Next step before the board: add Luca's existing cost base (current team,</t>
+          <t>over the 12 months), and I don't have the company's overall cost base: the model only includes the</t>
         </is>
       </c>
       <c r="C26" s="2" t="n"/>
@@ -1081,7 +1081,7 @@
       <c r="A27" s="2" t="n"/>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>marketing, technology) to the model. That is where runway and the loan decision become relevant.</t>
+          <t>25 new hires, overhead and G&amp;A.</t>
         </is>
       </c>
       <c r="C27" s="2" t="n"/>

</xml_diff>